<commit_message>
update script and katara deck
</commit_message>
<xml_diff>
--- a/katara_budget_plus_05_25_2026.xlsx
+++ b/katara_budget_plus_05_25_2026.xlsx
@@ -17,7 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$0.00"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -51,9 +53,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -445,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:J93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.86" customWidth="1" min="1" max="1"/>
@@ -453,8 +456,11 @@
     <col width="16.86" customWidth="1" min="3" max="3"/>
     <col width="16.86" customWidth="1" min="4" max="4"/>
     <col width="16.86" customWidth="1" min="5" max="5"/>
-    <col width="101.16" customWidth="1" min="6" max="6"/>
+    <col width="16.86" customWidth="1" min="6" max="6"/>
     <col width="16.86" customWidth="1" min="7" max="7"/>
+    <col width="16.86" customWidth="1" min="8" max="8"/>
+    <col width="101.16" customWidth="1" min="9" max="9"/>
+    <col width="16.86" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -485,10 +491,25 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Deck Rule</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Rarity</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>MTG Edition</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Image</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
@@ -512,11 +533,30 @@
         <v>0</v>
       </c>
       <c r="E2" t="inlineStr"/>
-      <c r="F2">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>TLA</t>
+        </is>
+      </c>
+      <c r="I2">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Katara%2C%20Water%20Tribe%27s%20Hope&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0.34$</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="270" customHeight="1">
       <c r="A3" t="inlineStr">
@@ -536,11 +576,30 @@
         <v>0</v>
       </c>
       <c r="E3" t="inlineStr"/>
-      <c r="F3">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>TLA</t>
+        </is>
+      </c>
+      <c r="I3">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Curious%20Farm%20Animals&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0.16$</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="270" customHeight="1">
       <c r="A4" t="inlineStr">
@@ -560,11 +619,30 @@
         <v>0</v>
       </c>
       <c r="E4" t="inlineStr"/>
-      <c r="F4">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>TLE</t>
+        </is>
+      </c>
+      <c r="I4">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Inspired%20Insurgent&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>0.12$</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="270" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -584,11 +662,30 @@
         <v>0</v>
       </c>
       <c r="E5" t="inlineStr"/>
-      <c r="F5">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>TLA</t>
+        </is>
+      </c>
+      <c r="I5">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Invasion%20Reinforcements&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>0.25$</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="270" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -608,11 +705,30 @@
         <v>0</v>
       </c>
       <c r="E6" t="inlineStr"/>
-      <c r="F6">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>CMM</t>
+        </is>
+      </c>
+      <c r="I6">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Ornithopter%20of%20Paradise&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>0.76$</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="270" customHeight="1">
       <c r="A7" t="inlineStr">
@@ -632,11 +748,30 @@
         <v>0</v>
       </c>
       <c r="E7" t="inlineStr"/>
-      <c r="F7">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>FDN</t>
+        </is>
+      </c>
+      <c r="I7">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Resolute%20Reinforcements&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>0.25$</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="270" customHeight="1">
       <c r="A8" t="inlineStr">
@@ -656,11 +791,30 @@
         <v>0</v>
       </c>
       <c r="E8" t="inlineStr"/>
-      <c r="F8">
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>CMM</t>
+        </is>
+      </c>
+      <c r="I8">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Tetsuko%20Umezawa%2C%20Fugitive&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>0.16$</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="270" customHeight="1">
       <c r="A9" t="inlineStr">
@@ -680,11 +834,30 @@
         <v>0</v>
       </c>
       <c r="E9" t="inlineStr"/>
-      <c r="F9">
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>TLA</t>
+        </is>
+      </c>
+      <c r="I9">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Earth%20Kingdom%20Jailer&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>0.21$</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="270" customHeight="1">
       <c r="A10" t="inlineStr">
@@ -704,11 +877,30 @@
         <v>0</v>
       </c>
       <c r="E10" t="inlineStr"/>
-      <c r="F10">
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>TLE</t>
+        </is>
+      </c>
+      <c r="I10">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Appa%2C%20Aang%27s%20Companion&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>0.37$</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="270" customHeight="1">
       <c r="A11" t="inlineStr">
@@ -728,11 +920,30 @@
         <v>0</v>
       </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11">
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>AKH</t>
+        </is>
+      </c>
+      <c r="I11">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Aven%20Wind%20Guide&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>0.31$</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="270" customHeight="1">
       <c r="A12" t="inlineStr">
@@ -752,11 +963,30 @@
         <v>0</v>
       </c>
       <c r="E12" t="inlineStr"/>
-      <c r="F12">
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Mythic</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>BLB</t>
+        </is>
+      </c>
+      <c r="I12">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Eluge%2C%20the%20Shoreless%20Sea&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>4.02$</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="270" customHeight="1">
       <c r="A13" t="inlineStr">
@@ -776,11 +1006,30 @@
         <v>0</v>
       </c>
       <c r="E13" t="inlineStr"/>
-      <c r="F13">
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>TDC</t>
+        </is>
+      </c>
+      <c r="I13">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Emeria%20Angel&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>0.36$</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="270" customHeight="1">
       <c r="A14" t="inlineStr">
@@ -800,11 +1049,30 @@
         <v>0</v>
       </c>
       <c r="E14" t="inlineStr"/>
-      <c r="F14">
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>MKC</t>
+        </is>
+      </c>
+      <c r="I14">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Keeper%20of%20the%20Accord&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>0.43$</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="270" customHeight="1">
       <c r="A15" t="inlineStr">
@@ -824,11 +1092,30 @@
         <v>0</v>
       </c>
       <c r="E15" t="inlineStr"/>
-      <c r="F15">
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>CMM</t>
+        </is>
+      </c>
+      <c r="I15">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Loyal%20Unicorn&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>0.24$</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="270" customHeight="1">
       <c r="A16" t="inlineStr">
@@ -848,11 +1135,30 @@
         <v>0</v>
       </c>
       <c r="E16" t="inlineStr"/>
-      <c r="F16">
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="I16">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Odric%2C%20Lunarch%20Marshal&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>1.12$</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="270" customHeight="1">
       <c r="A17" t="inlineStr">
@@ -872,11 +1178,30 @@
         <v>0</v>
       </c>
       <c r="E17" t="inlineStr"/>
-      <c r="F17">
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>TLA</t>
+        </is>
+      </c>
+      <c r="I17">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Appa%2C%20Loyal%20Sky%20Bison&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>0.31$</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="270" customHeight="1">
       <c r="A18" t="inlineStr">
@@ -896,11 +1221,30 @@
         <v>0</v>
       </c>
       <c r="E18" t="inlineStr"/>
-      <c r="F18">
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>EOC</t>
+        </is>
+      </c>
+      <c r="I18">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Threefold%20Thunderhulk&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>0.33$</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="270" customHeight="1">
       <c r="A19" t="inlineStr">
@@ -920,11 +1264,30 @@
         <v>0</v>
       </c>
       <c r="E19" t="inlineStr"/>
-      <c r="F19">
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Mythic</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>TLA</t>
+        </is>
+      </c>
+      <c r="I19">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=The%20Walls%20of%20Ba%20Sing%20Se&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>27.37$</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="270" customHeight="1">
       <c r="A20" t="inlineStr">
@@ -944,11 +1307,30 @@
         <v>0</v>
       </c>
       <c r="E20" t="inlineStr"/>
-      <c r="F20">
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Card Advantage</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>TDC</t>
+        </is>
+      </c>
+      <c r="I20">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Welcoming%20Vampire&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2.81$</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="270" customHeight="1">
       <c r="A21" t="inlineStr">
@@ -968,11 +1350,30 @@
         <v>0</v>
       </c>
       <c r="E21" t="inlineStr"/>
-      <c r="F21">
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Card Advantage</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>MKC</t>
+        </is>
+      </c>
+      <c r="I21">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Aerial%20Extortionist&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>4.07$</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="270" customHeight="1">
       <c r="A22" t="inlineStr">
@@ -992,11 +1393,30 @@
         <v>0</v>
       </c>
       <c r="E22" t="inlineStr"/>
-      <c r="F22">
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>TDC</t>
+        </is>
+      </c>
+      <c r="I22">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Adeline%2C%20Resplendent%20Cathar&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2.68$</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="270" customHeight="1">
       <c r="A23" t="inlineStr">
@@ -1016,11 +1436,30 @@
         <v>0</v>
       </c>
       <c r="E23" t="inlineStr"/>
-      <c r="F23">
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Card Advantage</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>SOC</t>
+        </is>
+      </c>
+      <c r="I23">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Curiosity%20Crafter&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>0.27$</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="270" customHeight="1">
       <c r="A24" t="inlineStr">
@@ -1040,11 +1479,30 @@
         <v>0</v>
       </c>
       <c r="E24" t="inlineStr"/>
-      <c r="F24">
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Card Advantage</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="I24">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Mentor%20of%20the%20Meek&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>0.40$</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="270" customHeight="1">
       <c r="A25" t="inlineStr">
@@ -1064,11 +1522,30 @@
         <v>0</v>
       </c>
       <c r="E25" t="inlineStr"/>
-      <c r="F25">
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>SOC</t>
+        </is>
+      </c>
+      <c r="I25">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Ajani%27s%20Chosen&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>0.26$</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="270" customHeight="1">
       <c r="A26" t="inlineStr">
@@ -1088,11 +1565,30 @@
         <v>0</v>
       </c>
       <c r="E26" t="inlineStr"/>
-      <c r="F26">
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>EOC</t>
+        </is>
+      </c>
+      <c r="I26">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Everflowing%20Chalice&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>0.35$</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="270" customHeight="1">
       <c r="A27" t="inlineStr">
@@ -1112,11 +1608,30 @@
         <v>0</v>
       </c>
       <c r="E27" t="inlineStr"/>
-      <c r="F27">
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Card Advantage</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>SOI</t>
+        </is>
+      </c>
+      <c r="I27">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Skeleton%20Key&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>0.35$</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="270" customHeight="1">
       <c r="A28" t="inlineStr">
@@ -1136,11 +1651,30 @@
         <v>0</v>
       </c>
       <c r="E28" t="inlineStr"/>
-      <c r="F28">
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>SOC</t>
+        </is>
+      </c>
+      <c r="I28">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Sol%20Ring&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>1.11$</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="270" customHeight="1">
       <c r="A29" t="inlineStr">
@@ -1160,11 +1694,30 @@
         <v>0</v>
       </c>
       <c r="E29" t="inlineStr"/>
-      <c r="F29">
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>TDC</t>
+        </is>
+      </c>
+      <c r="I29">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Wayfarer%27s%20Bauble&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>0.29$</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="270" customHeight="1">
       <c r="A30" t="inlineStr">
@@ -1184,11 +1737,30 @@
         <v>0</v>
       </c>
       <c r="E30" t="inlineStr"/>
-      <c r="F30">
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>SOC</t>
+        </is>
+      </c>
+      <c r="I30">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Arcane%20Signet&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>0.43$</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="270" customHeight="1">
       <c r="A31" t="inlineStr">
@@ -1208,11 +1780,30 @@
         <v>0</v>
       </c>
       <c r="E31" t="inlineStr"/>
-      <c r="F31">
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>TDC</t>
+        </is>
+      </c>
+      <c r="I31">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Azorius%20Signet&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>0.25$</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="270" customHeight="1">
       <c r="A32" t="inlineStr">
@@ -1232,11 +1823,30 @@
         <v>0</v>
       </c>
       <c r="E32" t="inlineStr"/>
-      <c r="F32">
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>SOC</t>
+        </is>
+      </c>
+      <c r="I32">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Mind%20Stone&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>0.33$</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="270" customHeight="1">
       <c r="A33" t="inlineStr">
@@ -1256,11 +1866,30 @@
         <v>0</v>
       </c>
       <c r="E33" t="inlineStr"/>
-      <c r="F33">
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>TDC</t>
+        </is>
+      </c>
+      <c r="I33">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Swiftfoot%20Boots&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2.22$</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="270" customHeight="1">
       <c r="A34" t="inlineStr">
@@ -1280,11 +1909,30 @@
         <v>0</v>
       </c>
       <c r="E34" t="inlineStr"/>
-      <c r="F34">
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>TDC</t>
+        </is>
+      </c>
+      <c r="I34">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Talisman%20of%20Progress&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>0.37$</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="270" customHeight="1">
       <c r="A35" t="inlineStr">
@@ -1304,11 +1952,30 @@
         <v>0</v>
       </c>
       <c r="E35" t="inlineStr"/>
-      <c r="F35">
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>DSC</t>
+        </is>
+      </c>
+      <c r="I35">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Thought%20Vessel&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2.61$</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="270" customHeight="1">
       <c r="A36" t="inlineStr">
@@ -1328,11 +1995,30 @@
         <v>0</v>
       </c>
       <c r="E36" t="inlineStr"/>
-      <c r="F36">
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>SOC</t>
+        </is>
+      </c>
+      <c r="I36">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Archaeomancer%27s%20Map&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>1.29$</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="270" customHeight="1">
       <c r="A37" t="inlineStr">
@@ -1352,11 +2038,30 @@
         <v>0</v>
       </c>
       <c r="E37" t="inlineStr"/>
-      <c r="F37">
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>FDN</t>
+        </is>
+      </c>
+      <c r="I37">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Hedron%20Archive&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>0.18$</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="270" customHeight="1">
       <c r="A38" t="inlineStr">
@@ -1376,11 +2081,30 @@
         <v>0</v>
       </c>
       <c r="E38" t="inlineStr"/>
-      <c r="F38">
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Card Advantage</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>TDC</t>
+        </is>
+      </c>
+      <c r="I38">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Idol%20of%20Oblivion&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>0.99$</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="270" customHeight="1">
       <c r="A39" t="inlineStr">
@@ -1400,11 +2124,30 @@
         <v>0</v>
       </c>
       <c r="E39" t="inlineStr"/>
-      <c r="F39">
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>CMM</t>
+        </is>
+      </c>
+      <c r="I39">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Thran%20Dynamo&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>4.08$</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="270" customHeight="1">
       <c r="A40" t="inlineStr">
@@ -1424,11 +2167,30 @@
         <v>0</v>
       </c>
       <c r="E40" t="inlineStr"/>
-      <c r="F40">
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>FDN</t>
+        </is>
+      </c>
+      <c r="I40">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Gilded%20Lotus&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>0.47$</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="270" customHeight="1">
       <c r="A41" t="inlineStr">
@@ -1448,11 +2210,30 @@
         <v>0</v>
       </c>
       <c r="E41" t="inlineStr"/>
-      <c r="F41">
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>CMD</t>
+        </is>
+      </c>
+      <c r="I41">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Journey%20to%20Nowhere&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>0.47$</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="270" customHeight="1">
       <c r="A42" t="inlineStr">
@@ -1472,11 +2253,30 @@
         <v>0</v>
       </c>
       <c r="E42" t="inlineStr"/>
-      <c r="F42">
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>TMT</t>
+        </is>
+      </c>
+      <c r="I42">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Uneasy%20Alliance&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>0.11$</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="270" customHeight="1">
       <c r="A43" t="inlineStr">
@@ -1496,11 +2296,30 @@
         <v>0</v>
       </c>
       <c r="E43" t="inlineStr"/>
-      <c r="F43">
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>EOE</t>
+        </is>
+      </c>
+      <c r="I43">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Banishing%20Light&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>0.19$</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="270" customHeight="1">
       <c r="A44" t="inlineStr">
@@ -1520,11 +2339,30 @@
         <v>0</v>
       </c>
       <c r="E44" t="inlineStr"/>
-      <c r="F44">
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Card Advantage</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>JMP</t>
+        </is>
+      </c>
+      <c r="I44">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Coastal%20Piracy&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>0.92$</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="270" customHeight="1">
       <c r="A45" t="inlineStr">
@@ -1544,11 +2382,30 @@
         <v>0</v>
       </c>
       <c r="E45" t="inlineStr"/>
-      <c r="F45">
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Wrath</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>DSK</t>
+        </is>
+      </c>
+      <c r="I45">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Restricted%20Office%20%2F%2F%20Lecture%20Hall&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>0.18$</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="270" customHeight="1">
       <c r="A46" t="inlineStr">
@@ -1568,11 +2425,30 @@
         <v>0</v>
       </c>
       <c r="E46" t="inlineStr"/>
-      <c r="F46">
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Card Advantage</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="I46">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Reconnaissance%20Mission&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>1.50$</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="270" customHeight="1">
       <c r="A47" t="inlineStr">
@@ -1592,11 +2468,30 @@
         <v>0</v>
       </c>
       <c r="E47" t="inlineStr"/>
-      <c r="F47">
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Card Advantage</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>SOC</t>
+        </is>
+      </c>
+      <c r="I47">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Tocasia%27s%20Welcome&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>0.58$</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="270" customHeight="1">
       <c r="A48" t="inlineStr">
@@ -1616,11 +2511,30 @@
         <v>0</v>
       </c>
       <c r="E48" t="inlineStr"/>
-      <c r="F48">
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Card Advantage</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>ZNC</t>
+        </is>
+      </c>
+      <c r="I48">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Military%20Intelligence&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>0.36$</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="270" customHeight="1">
       <c r="A49" t="inlineStr">
@@ -1640,11 +2554,30 @@
         <v>0</v>
       </c>
       <c r="E49" t="inlineStr"/>
-      <c r="F49">
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>SOC</t>
+        </is>
+      </c>
+      <c r="I49">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Path%20to%20Exile&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>0.99$</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="270" customHeight="1">
       <c r="A50" t="inlineStr">
@@ -1664,11 +2597,30 @@
         <v>0</v>
       </c>
       <c r="E50" t="inlineStr"/>
-      <c r="F50">
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>TLA</t>
+        </is>
+      </c>
+      <c r="I50">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Airbender%27s%20Reversal&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>0.26$</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="270" customHeight="1">
       <c r="A51" t="inlineStr">
@@ -1688,11 +2640,30 @@
         <v>0</v>
       </c>
       <c r="E51" t="inlineStr"/>
-      <c r="F51">
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>SOS</t>
+        </is>
+      </c>
+      <c r="I51">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Essence%20Scatter&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>0.20$</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="270" customHeight="1">
       <c r="A52" t="inlineStr">
@@ -1712,11 +2683,30 @@
         <v>0</v>
       </c>
       <c r="E52" t="inlineStr"/>
-      <c r="F52">
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>TMT</t>
+        </is>
+      </c>
+      <c r="I52">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Negate&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>0.27$</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="270" customHeight="1">
       <c r="A53" t="inlineStr">
@@ -1736,11 +2726,30 @@
         <v>0</v>
       </c>
       <c r="E53" t="inlineStr"/>
-      <c r="F53">
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>TDC</t>
+        </is>
+      </c>
+      <c r="I53">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Stroke%20of%20Midnight&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>0.34$</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="270" customHeight="1">
       <c r="A54" t="inlineStr">
@@ -1760,11 +2769,30 @@
         <v>0</v>
       </c>
       <c r="E54" t="inlineStr"/>
-      <c r="F54">
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>CMR</t>
+        </is>
+      </c>
+      <c r="I54">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=White%20Sun%27s%20Zenith&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>0.32$</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="270" customHeight="1">
       <c r="A55" t="inlineStr">
@@ -1784,11 +2812,30 @@
         <v>0</v>
       </c>
       <c r="E55" t="inlineStr"/>
-      <c r="F55">
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>TMT</t>
+        </is>
+      </c>
+      <c r="I55">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=The%20Last%20Ronin%27s%20Technique&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>0.25$</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="270" customHeight="1">
       <c r="A56" t="inlineStr">
@@ -1808,11 +2855,30 @@
         <v>0</v>
       </c>
       <c r="E56" t="inlineStr"/>
-      <c r="F56">
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>LCC</t>
+        </is>
+      </c>
+      <c r="I56">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Generous%20Gift&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G56" t="inlineStr"/>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>1.62$</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="270" customHeight="1">
       <c r="A57" t="inlineStr">
@@ -1832,11 +2898,30 @@
         <v>0</v>
       </c>
       <c r="E57" t="inlineStr"/>
-      <c r="F57">
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>SOC</t>
+        </is>
+      </c>
+      <c r="I57">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Swords%20to%20Plowshares&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>1.33$</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="270" customHeight="1">
       <c r="A58" t="inlineStr">
@@ -1856,11 +2941,30 @@
         <v>0</v>
       </c>
       <c r="E58" t="inlineStr"/>
-      <c r="F58">
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>MOC</t>
+        </is>
+      </c>
+      <c r="I58">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Path%20of%20the%20Ghosthunter&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G58" t="inlineStr"/>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>0.30$</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="270" customHeight="1">
       <c r="A59" t="inlineStr">
@@ -1880,11 +2984,30 @@
         <v>0</v>
       </c>
       <c r="E59" t="inlineStr"/>
-      <c r="F59">
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Wrath</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>LTR</t>
+        </is>
+      </c>
+      <c r="I59">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=The%20Battle%20of%20Bywater&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G59" t="inlineStr"/>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>3.08$</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="270" customHeight="1">
       <c r="A60" t="inlineStr">
@@ -1904,11 +3027,30 @@
         <v>0</v>
       </c>
       <c r="E60" t="inlineStr"/>
-      <c r="F60">
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>MH3</t>
+        </is>
+      </c>
+      <c r="I60">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Decree%20of%20Justice&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>0.27$</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="270" customHeight="1">
       <c r="A61" t="inlineStr">
@@ -1928,11 +3070,30 @@
         <v>0</v>
       </c>
       <c r="E61" t="inlineStr"/>
-      <c r="F61">
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Wrath</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>TDC</t>
+        </is>
+      </c>
+      <c r="I61">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Expel%20the%20Interlopers&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>0.28$</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="270" customHeight="1">
       <c r="A62" t="inlineStr">
@@ -1952,11 +3113,30 @@
         <v>0</v>
       </c>
       <c r="E62" t="inlineStr"/>
-      <c r="F62">
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Wrath</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>MKC</t>
+        </is>
+      </c>
+      <c r="I62">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Fell%20the%20Mighty&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>0.22$</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="270" customHeight="1">
       <c r="A63" t="inlineStr">
@@ -1976,11 +3156,30 @@
         <v>0</v>
       </c>
       <c r="E63" t="inlineStr"/>
-      <c r="F63">
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Wrath</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>MKC</t>
+        </is>
+      </c>
+      <c r="I63">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Dusk%20%2F%2F%20Dawn&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>0.32$</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="270" customHeight="1">
       <c r="A64" t="inlineStr">
@@ -2000,11 +3199,30 @@
         <v>0</v>
       </c>
       <c r="E64" t="inlineStr"/>
-      <c r="F64">
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>EOC</t>
+        </is>
+      </c>
+      <c r="I64">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Glacial%20Fortress&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>0.33$</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="270" customHeight="1">
       <c r="A65" t="inlineStr">
@@ -2024,11 +3242,30 @@
         <v>0</v>
       </c>
       <c r="E65" t="inlineStr"/>
-      <c r="F65">
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>DMU</t>
+        </is>
+      </c>
+      <c r="I65">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Idyllic%20Beachfront&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G65" t="inlineStr"/>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>0.26$</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="270" customHeight="1">
       <c r="A66" t="inlineStr">
@@ -2048,11 +3285,30 @@
         <v>0</v>
       </c>
       <c r="E66" t="inlineStr"/>
-      <c r="F66">
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>EOC</t>
+        </is>
+      </c>
+      <c r="I66">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Irrigated%20Farmland&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>0.17$</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="270" customHeight="1">
       <c r="A67" t="inlineStr">
@@ -2072,11 +3328,26 @@
         <v>0</v>
       </c>
       <c r="E67" t="inlineStr"/>
-      <c r="F67">
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>HOB</t>
+        </is>
+      </c>
+      <c r="I67">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Island&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
     </row>
     <row r="68" ht="270" customHeight="1">
       <c r="A68" t="inlineStr">
@@ -2096,11 +3367,30 @@
         <v>0</v>
       </c>
       <c r="E68" t="inlineStr"/>
-      <c r="F68">
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>TLA</t>
+        </is>
+      </c>
+      <c r="I68">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=North%20Pole%20Gates&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G68" t="inlineStr"/>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>0.24$</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="270" customHeight="1">
       <c r="A69" t="inlineStr">
@@ -2120,11 +3410,26 @@
         <v>0</v>
       </c>
       <c r="E69" t="inlineStr"/>
-      <c r="F69">
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>HOB</t>
+        </is>
+      </c>
+      <c r="I69">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Plains&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
     </row>
     <row r="70" ht="270" customHeight="1">
       <c r="A70" t="inlineStr">
@@ -2144,11 +3449,30 @@
         <v>0</v>
       </c>
       <c r="E70" t="inlineStr"/>
-      <c r="F70">
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>CMM</t>
+        </is>
+      </c>
+      <c r="I70">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Port%20Town&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G70" t="inlineStr"/>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>0.22$</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="270" customHeight="1">
       <c r="A71" t="inlineStr">
@@ -2168,11 +3492,30 @@
         <v>0</v>
       </c>
       <c r="E71" t="inlineStr"/>
-      <c r="F71">
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>TDC</t>
+        </is>
+      </c>
+      <c r="I71">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Prairie%20Stream&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G71" t="inlineStr"/>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>0.26$</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="270" customHeight="1">
       <c r="A72" t="inlineStr">
@@ -2192,11 +3535,30 @@
         <v>0</v>
       </c>
       <c r="E72" t="inlineStr"/>
-      <c r="F72">
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>EOC</t>
+        </is>
+      </c>
+      <c r="I72">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Skycloud%20Expanse&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G72" t="inlineStr"/>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>0.27$</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="270" customHeight="1">
       <c r="A73" t="inlineStr">
@@ -2216,11 +3578,30 @@
         <v>0</v>
       </c>
       <c r="E73" t="inlineStr"/>
-      <c r="F73">
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>EOC</t>
+        </is>
+      </c>
+      <c r="I73">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Temple%20of%20Enlightenment&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G73" t="inlineStr"/>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>0.26$</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="270" customHeight="1">
       <c r="A74" t="inlineStr">
@@ -2240,11 +3621,30 @@
         <v>0</v>
       </c>
       <c r="E74" t="inlineStr"/>
-      <c r="F74">
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>ECC</t>
+        </is>
+      </c>
+      <c r="I74">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Thriving%20Heath&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G74" t="inlineStr"/>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>0.23$</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="270" customHeight="1">
       <c r="A75" t="inlineStr">
@@ -2264,11 +3664,30 @@
         <v>0</v>
       </c>
       <c r="E75" t="inlineStr"/>
-      <c r="F75">
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>TMC</t>
+        </is>
+      </c>
+      <c r="I75">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Thriving%20Isle&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G75" t="inlineStr"/>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>0.29$</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="270" customHeight="1">
       <c r="A76" t="inlineStr">
@@ -2288,11 +3707,30 @@
         <v>0</v>
       </c>
       <c r="E76" t="inlineStr"/>
-      <c r="F76">
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Lands</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>SOC</t>
+        </is>
+      </c>
+      <c r="I76">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Command%20Tower&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G76" t="inlineStr"/>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>0.34$</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="270" customHeight="1">
       <c r="A77" t="inlineStr">
@@ -2314,11 +3752,30 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F77">
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>ECL</t>
+        </is>
+      </c>
+      <c r="I77">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Stalactite%20Dagger&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G77" t="inlineStr"/>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>0.23$</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="270" customHeight="1">
       <c r="A78" t="inlineStr">
@@ -2340,11 +3797,30 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F78">
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>FIN</t>
+        </is>
+      </c>
+      <c r="I78">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Magitek%20Armor&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G78" t="inlineStr"/>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>0.06$</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="270" customHeight="1">
       <c r="A79" t="inlineStr">
@@ -2366,11 +3842,30 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F79">
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>TDM</t>
+        </is>
+      </c>
+      <c r="I79">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Stormbeacon%20Blade&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G79" t="inlineStr"/>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>0.25$</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="270" customHeight="1">
       <c r="A80" t="inlineStr">
@@ -2392,11 +3887,30 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F80">
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>FDN</t>
+        </is>
+      </c>
+      <c r="I80">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Guarded%20Heir&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G80" t="inlineStr"/>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>0.11$</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="270" customHeight="1">
       <c r="A81" t="inlineStr">
@@ -2418,11 +3932,30 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F81">
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>TLA</t>
+        </is>
+      </c>
+      <c r="I81">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Kyoshi%20Warriors&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G81" t="inlineStr"/>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>0.12$</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="270" customHeight="1">
       <c r="A82" t="inlineStr">
@@ -2444,11 +3977,30 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F82">
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>TLA</t>
+        </is>
+      </c>
+      <c r="I82">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Gather%20the%20White%20Lotus&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G82" t="inlineStr"/>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>0.15$</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="270" customHeight="1">
       <c r="A83" t="inlineStr">
@@ -2470,11 +4022,30 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F83">
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>LCC</t>
+        </is>
+      </c>
+      <c r="I83">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=March%20of%20the%20Canonized&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G83" t="inlineStr"/>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>0.31$</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="270" customHeight="1">
       <c r="A84" t="inlineStr">
@@ -2496,11 +4067,30 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F84">
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>TDC</t>
+        </is>
+      </c>
+      <c r="I84">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Release%20the%20Dogs&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G84" t="inlineStr"/>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>0.34$</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="270" customHeight="1">
       <c r="A85" t="inlineStr">
@@ -2522,11 +4112,30 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F85">
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>OTC</t>
+        </is>
+      </c>
+      <c r="I85">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Prismatic%20Lens&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G85" t="inlineStr"/>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>0.41$</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="270" customHeight="1">
       <c r="A86" t="inlineStr">
@@ -2548,11 +4157,30 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F86">
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>DSK</t>
+        </is>
+      </c>
+      <c r="I86">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Cursed%20Windbreaker&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G86" t="inlineStr"/>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>0.16$</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="270" customHeight="1">
       <c r="A87" t="inlineStr">
@@ -2574,11 +4202,30 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F87">
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>TLA</t>
+        </is>
+      </c>
+      <c r="I87">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Fire%20Nation%20Warship&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G87" t="inlineStr"/>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>0.13$</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="270" customHeight="1">
       <c r="A88" t="inlineStr">
@@ -2600,11 +4247,30 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F88">
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Card Advantage</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>SOS</t>
+        </is>
+      </c>
+      <c r="I88">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Quick%20Study&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G88" t="inlineStr"/>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>0.18$</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="270" customHeight="1">
       <c r="A89" t="inlineStr">
@@ -2626,11 +4292,30 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F89">
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>FDN</t>
+        </is>
+      </c>
+      <c r="I89">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Refute&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G89" t="inlineStr"/>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>0.29$</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="270" customHeight="1">
       <c r="A90" t="inlineStr">
@@ -2652,11 +4337,30 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F90">
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>FIN</t>
+        </is>
+      </c>
+      <c r="I90">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=The%20Crystal%27s%20Chosen&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G90" t="inlineStr"/>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>0.15$</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="270" customHeight="1">
       <c r="A91" t="inlineStr">
@@ -2678,11 +4382,41 @@
           <t>Trimmed low-impact equipment and one-shot/low-impact spells to add repeatable draw engines and explosive ramp.</t>
         </is>
       </c>
-      <c r="F91">
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>On Theme</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Uncommon</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>TLA</t>
+        </is>
+      </c>
+      <c r="I91">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Team%20Avatar&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="G91" t="inlineStr"/>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>0.18$</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Total Cost (Have Physical Copy = false)</t>
+        </is>
+      </c>
+      <c r="J93" s="2">
+        <f>SUMPRODUCT(--(LOWER(TEXT($C$2:$C$91,"@"))="false"),IFERROR(VALUE(SUBSTITUTE($J$2:$J$91,"$","")),0))</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C91">

</xml_diff>

<commit_message>
add mana value and oracle text
</commit_message>
<xml_diff>
--- a/katara_budget_plus_05_25_2026.xlsx
+++ b/katara_budget_plus_05_25_2026.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J93"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.86" customWidth="1" min="1" max="1"/>
@@ -459,8 +459,10 @@
     <col width="16.86" customWidth="1" min="6" max="6"/>
     <col width="16.86" customWidth="1" min="7" max="7"/>
     <col width="16.86" customWidth="1" min="8" max="8"/>
-    <col width="101.16" customWidth="1" min="9" max="9"/>
-    <col width="16.86" customWidth="1" min="10" max="10"/>
+    <col width="16.86" customWidth="1" min="9" max="9"/>
+    <col width="101.16" customWidth="1" min="10" max="10"/>
+    <col width="16.86" customWidth="1" min="11" max="11"/>
+    <col width="16.86" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,12 +508,22 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Mana Value</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Image</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Price</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Rule Text</t>
         </is>
       </c>
     </row>
@@ -548,13 +560,25 @@
           <t>TLA</t>
         </is>
       </c>
-      <c r="I2">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J2">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Katara%2C%20Water%20Tribe%27s%20Hope&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>0.34$</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Vigilance
+When Katara enters, create a 1/1 white Ally creature token.
+Waterbend {X}: Creatures you control have base power and toughness X/X until end of turn. X can't be 0. Activate only during your turn. (While paying a waterbend cost, you can tap your artifacts and creatures to help. Each one pays for {1}.)</t>
         </is>
       </c>
     </row>
@@ -591,13 +615,24 @@
           <t>TLA</t>
         </is>
       </c>
-      <c r="I3">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J3">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Curious%20Farm%20Animals&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>0.16$</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>When this creature dies, you gain 3 life.
+{2}, Sacrifice this creature: Destroy up to one target artifact or enchantment.</t>
         </is>
       </c>
     </row>
@@ -634,13 +669,23 @@
           <t>TLE</t>
         </is>
       </c>
-      <c r="I4">
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J4">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Inspired%20Insurgent&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>0.12$</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>{1}, Sacrifice this creature: Destroy target artifact or enchantment.</t>
         </is>
       </c>
     </row>
@@ -677,13 +722,24 @@
           <t>TLA</t>
         </is>
       </c>
-      <c r="I5">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J5">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Invasion%20Reinforcements&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>0.25$</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Flash
+When this creature enters, create a 1/1 white Ally creature token.</t>
         </is>
       </c>
     </row>
@@ -720,13 +776,24 @@
           <t>CMM</t>
         </is>
       </c>
-      <c r="I6">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J6">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Ornithopter%20of%20Paradise&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>0.76$</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Flying
+{T}: Add one mana of any color.</t>
         </is>
       </c>
     </row>
@@ -763,13 +830,24 @@
           <t>FDN</t>
         </is>
       </c>
-      <c r="I7">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J7">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Resolute%20Reinforcements&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>0.25$</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Flash (You may cast this spell any time you could cast an instant.)
+When this creature enters, create a 1/1 white Soldier creature token.</t>
         </is>
       </c>
     </row>
@@ -806,13 +884,23 @@
           <t>CMM</t>
         </is>
       </c>
-      <c r="I8">
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J8">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Tetsuko%20Umezawa%2C%20Fugitive&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>0.16$</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Creatures you control with power or toughness 1 or less can't be blocked.</t>
         </is>
       </c>
     </row>
@@ -849,13 +937,23 @@
           <t>TLA</t>
         </is>
       </c>
-      <c r="I9">
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J9">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Earth%20Kingdom%20Jailer&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>0.21$</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>When this creature enters, exile up to one target artifact, creature, or enchantment an opponent controls with mana value 3 or greater until this creature leaves the battlefield.</t>
         </is>
       </c>
     </row>
@@ -892,13 +990,24 @@
           <t>TLE</t>
         </is>
       </c>
-      <c r="I10">
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J10">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Appa%2C%20Aang%27s%20Companion&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>0.37$</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Flying (This creature can't be blocked except by creatures with flying or reach.)
+Whenever Appa attacks, another target attacking creature without flying gains flying until end of turn.</t>
         </is>
       </c>
     </row>
@@ -935,13 +1044,25 @@
           <t>AKH</t>
         </is>
       </c>
-      <c r="I11">
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J11">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Aven%20Wind%20Guide&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>0.31$</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Flying, vigilance
+Creature tokens you control have flying and vigilance.
+Embalm {4}{W}{U} ({4}{W}{U}, Exile this card from your graveyard: Create a token that's a copy of it, except it's a white Zombie Bird Warrior with no mana cost. Embalm only as a sorcery.)</t>
         </is>
       </c>
     </row>
@@ -978,13 +1099,25 @@
           <t>BLB</t>
         </is>
       </c>
-      <c r="I12">
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J12">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Eluge%2C%20the%20Shoreless%20Sea&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>4.02$</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Eluge's power and toughness are each equal to the number of Islands you control.
+Whenever Eluge enters or attacks, put a flood counter on target land. It's an Island in addition to its other types for as long as it has a flood counter on it.
+The first instant or sorcery spell you cast each turn costs {U} (or {1}) less to cast for each land you control with a flood counter on it.</t>
         </is>
       </c>
     </row>
@@ -1021,13 +1154,24 @@
           <t>TDC</t>
         </is>
       </c>
-      <c r="I13">
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J13">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Emeria%20Angel&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>0.36$</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Flying
+Landfall - Whenever a land you control enters, you may create a 1/1 white Bird creature token with flying.</t>
         </is>
       </c>
     </row>
@@ -1064,13 +1208,24 @@
           <t>MKC</t>
         </is>
       </c>
-      <c r="I14">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J14">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Keeper%20of%20the%20Accord&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>0.43$</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>At the beginning of each opponent's end step, if that player controls more creatures than you, create a 1/1 white Soldier creature token.
+At the beginning of each opponent's end step, if that player controls more lands than you, you may search your library for a basic Plains card, put it onto the battlefield tapped, then shuffle.</t>
         </is>
       </c>
     </row>
@@ -1107,13 +1262,24 @@
           <t>CMM</t>
         </is>
       </c>
-      <c r="I15">
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J15">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Loyal%20Unicorn&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>0.24$</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Vigilance
+Lieutenant - At the beginning of combat on your turn, if you control your commander, prevent all combat damage that would be dealt to creatures you control this turn. Other creatures you control gain vigilance until end of turn.</t>
         </is>
       </c>
     </row>
@@ -1150,13 +1316,23 @@
           <t>INR</t>
         </is>
       </c>
-      <c r="I16">
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J16">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Odric%2C%20Lunarch%20Marshal&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>1.12$</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>At the beginning of each combat, creatures you control gain first strike until end of turn if a creature you control has first strike. The same is true for flying, deathtouch, double strike, haste, hexproof, indestructible, lifelink, menace, reach, skulk, trample, and vigilance.</t>
         </is>
       </c>
     </row>
@@ -1193,13 +1369,26 @@
           <t>TLA</t>
         </is>
       </c>
-      <c r="I17">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="J17">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Appa%2C%20Loyal%20Sky%20Bison&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>0.31$</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Flying
+Whenever Appa enters or attacks, choose one -
+- Target creature you control gains flying until end of turn.
+- Airbend another target nonland permanent you control. (Exile it. While it's exiled, its owner may cast it for {2} rather than its mana cost.)</t>
         </is>
       </c>
     </row>
@@ -1236,13 +1425,25 @@
           <t>EOC</t>
         </is>
       </c>
-      <c r="I18">
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="J18">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Threefold%20Thunderhulk&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>0.33$</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>This creature enters with three +1/+1 counters on it.
+Whenever this creature enters or attacks, create a number of 1/1 colorless Gnome artifact creature tokens equal to its power.
+{2}, Sacrifice another artifact: Put a +1/+1 counter on this creature.</t>
         </is>
       </c>
     </row>
@@ -1279,13 +1480,24 @@
           <t>TLA</t>
         </is>
       </c>
-      <c r="I19">
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="J19">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=The%20Walls%20of%20Ba%20Sing%20Se&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>27.37$</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Defender
+Other permanents you control have indestructible.</t>
         </is>
       </c>
     </row>
@@ -1322,13 +1534,24 @@
           <t>TDC</t>
         </is>
       </c>
-      <c r="I20">
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J20">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Welcoming%20Vampire&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>2.81$</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Flying
+Whenever one or more other creatures you control with power 2 or less enter, draw a card. This ability triggers only once each turn.</t>
         </is>
       </c>
     </row>
@@ -1365,13 +1588,25 @@
           <t>MKC</t>
         </is>
       </c>
-      <c r="I21">
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J21">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Aerial%20Extortionist&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>4.07$</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Flying
+Whenever this creature enters or deals combat damage to a player, exile up to one target nonland permanent. For as long as that card remains exiled, its owner may cast it.
+Whenever another player casts a spell from anywhere other than their hand, draw a card.</t>
         </is>
       </c>
     </row>
@@ -1408,13 +1643,25 @@
           <t>TDC</t>
         </is>
       </c>
-      <c r="I22">
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J22">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Adeline%2C%20Resplendent%20Cathar&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>2.68$</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Vigilance
+Adeline's power is equal to the number of creatures you control.
+Whenever you attack, for each opponent, create a 1/1 white Human creature token that's tapped and attacking that player or a planeswalker they control.</t>
         </is>
       </c>
     </row>
@@ -1451,13 +1698,25 @@
           <t>SOC</t>
         </is>
       </c>
-      <c r="I23">
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J23">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Curiosity%20Crafter&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>0.27$</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Flying
+You have no maximum hand size.
+Whenever a creature token you control deals combat damage to a player, draw a card.</t>
         </is>
       </c>
     </row>
@@ -1494,13 +1753,23 @@
           <t>INR</t>
         </is>
       </c>
-      <c r="I24">
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J24">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Mentor%20of%20the%20Meek&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>0.40$</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Whenever another creature you control with power 2 or less enters, you may pay {1}. If you do, draw a card.</t>
         </is>
       </c>
     </row>
@@ -1537,13 +1806,23 @@
           <t>SOC</t>
         </is>
       </c>
-      <c r="I25">
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J25">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Ajani%27s%20Chosen&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>0.26$</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Whenever an enchantment you control enters, create a 2/2 white Cat creature token. If that enchantment is an Aura, you may attach it to the token.</t>
         </is>
       </c>
     </row>
@@ -1580,13 +1859,25 @@
           <t>EOC</t>
         </is>
       </c>
-      <c r="I26">
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J26">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Everflowing%20Chalice&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>0.35$</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Multikicker {2} (You may pay an additional {2} any number of times as you cast this spell.)
+This artifact enters with a charge counter on it for each time it was kicked.
+{T}: Add {C} for each charge counter on this artifact.</t>
         </is>
       </c>
     </row>
@@ -1623,13 +1914,25 @@
           <t>SOI</t>
         </is>
       </c>
-      <c r="I27">
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J27">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Skeleton%20Key&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>0.35$</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Equipped creature has skulk. (It can't be blocked by creatures with greater power.)
+Whenever equipped creature deals combat damage to a player, you may draw a card. If you do, discard a card.
+Equip {2}</t>
         </is>
       </c>
     </row>
@@ -1666,13 +1969,23 @@
           <t>SOC</t>
         </is>
       </c>
-      <c r="I28">
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J28">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Sol%20Ring&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>1.11$</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>{T}: Add {C}{C}.</t>
         </is>
       </c>
     </row>
@@ -1709,13 +2022,23 @@
           <t>TDC</t>
         </is>
       </c>
-      <c r="I29">
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J29">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Wayfarer%27s%20Bauble&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>0.29$</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>{2}, {T}, Sacrifice this artifact: Search your library for a basic land card, put that card onto the battlefield tapped, then shuffle.</t>
         </is>
       </c>
     </row>
@@ -1752,13 +2075,23 @@
           <t>SOC</t>
         </is>
       </c>
-      <c r="I30">
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J30">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Arcane%20Signet&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>0.43$</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>{T}: Add one mana of any color in your commander's color identity.</t>
         </is>
       </c>
     </row>
@@ -1795,13 +2128,23 @@
           <t>TDC</t>
         </is>
       </c>
-      <c r="I31">
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J31">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Azorius%20Signet&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>0.25$</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>{1}, {T}: Add {W}{U}.</t>
         </is>
       </c>
     </row>
@@ -1838,13 +2181,24 @@
           <t>SOC</t>
         </is>
       </c>
-      <c r="I32">
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J32">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Mind%20Stone&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>0.33$</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>{T}: Add {C}.
+{1}, {T}, Sacrifice this artifact: Draw a card.</t>
         </is>
       </c>
     </row>
@@ -1881,13 +2235,24 @@
           <t>TDC</t>
         </is>
       </c>
-      <c r="I33">
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J33">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Swiftfoot%20Boots&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>2.22$</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Equipped creature has hexproof and haste. (It can't be the target of spells or abilities your opponents control. It can attack and {T} no matter when it came under your control.)
+Equip {1} ({1}: Attach to target creature you control. Equip only as a sorcery.)</t>
         </is>
       </c>
     </row>
@@ -1924,13 +2289,24 @@
           <t>TDC</t>
         </is>
       </c>
-      <c r="I34">
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J34">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Talisman%20of%20Progress&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>0.37$</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>{T}: Add {C}.
+{T}: Add {W} or {U}. This artifact deals 1 damage to you.</t>
         </is>
       </c>
     </row>
@@ -1967,13 +2343,24 @@
           <t>DSC</t>
         </is>
       </c>
-      <c r="I35">
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J35">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Thought%20Vessel&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>2.61$</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>You have no maximum hand size.
+{T}: Add {C}.</t>
         </is>
       </c>
     </row>
@@ -2010,13 +2397,24 @@
           <t>SOC</t>
         </is>
       </c>
-      <c r="I36">
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J36">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Archaeomancer%27s%20Map&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>1.29$</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>When this artifact enters, search your library for up to two basic Plains cards, reveal them, put them into your hand, then shuffle.
+Whenever a land an opponent controls enters, if that player controls more lands than you, you may put a land card from your hand onto the battlefield.</t>
         </is>
       </c>
     </row>
@@ -2053,13 +2451,24 @@
           <t>FDN</t>
         </is>
       </c>
-      <c r="I37">
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J37">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Hedron%20Archive&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>0.18$</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>{T}: Add {C}{C}.
+{2}, {T}, Sacrifice this artifact: Draw two cards.</t>
         </is>
       </c>
     </row>
@@ -2096,13 +2505,24 @@
           <t>TDC</t>
         </is>
       </c>
-      <c r="I38">
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J38">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Idol%20of%20Oblivion&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>0.99$</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>{T}: Draw a card. Activate only if you created a token this turn.
+{8}, {T}, Sacrifice this artifact: Create a 10/10 colorless Eldrazi creature token.</t>
         </is>
       </c>
     </row>
@@ -2139,13 +2559,23 @@
           <t>CMM</t>
         </is>
       </c>
-      <c r="I39">
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J39">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Thran%20Dynamo&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>4.08$</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>{T}: Add {C}{C}{C}.</t>
         </is>
       </c>
     </row>
@@ -2182,13 +2612,23 @@
           <t>FDN</t>
         </is>
       </c>
-      <c r="I40">
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J40">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Gilded%20Lotus&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>0.47$</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>{T}: Add three mana of any one color.</t>
         </is>
       </c>
     </row>
@@ -2225,13 +2665,24 @@
           <t>CMD</t>
         </is>
       </c>
-      <c r="I41">
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J41">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Journey%20to%20Nowhere&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>0.47$</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>When this enchantment enters, exile target creature.
+When this enchantment leaves the battlefield, return the exiled card to the battlefield under its owner's control.</t>
         </is>
       </c>
     </row>
@@ -2268,13 +2719,25 @@
           <t>TMT</t>
         </is>
       </c>
-      <c r="I42">
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J42">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Uneasy%20Alliance&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>0.11$</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Enchant creature
+Enchanted creature can't attack or block.
+{5}, Sacrifice this Aura: Exile enchanted creature. You create a 1/1 black Ninja creature token. Activate only as a sorcery.</t>
         </is>
       </c>
     </row>
@@ -2311,13 +2774,23 @@
           <t>EOE</t>
         </is>
       </c>
-      <c r="I43">
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J43">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Banishing%20Light&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>0.19$</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>When this enchantment enters, exile target nonland permanent an opponent controls until this enchantment leaves the battlefield.</t>
         </is>
       </c>
     </row>
@@ -2354,13 +2827,23 @@
           <t>JMP</t>
         </is>
       </c>
-      <c r="I44">
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J44">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Coastal%20Piracy&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>0.92$</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Whenever a creature you control deals combat damage to an opponent, you may draw a card.</t>
         </is>
       </c>
     </row>
@@ -2397,13 +2880,25 @@
           <t>DSK</t>
         </is>
       </c>
-      <c r="I45">
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="J45">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Restricted%20Office%20%2F%2F%20Lecture%20Hall&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>0.18$</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>When you unlock this door, destroy all creatures with power 3 or greater.
+(You may cast either half. That door unlocks on the battlefield. As a sorcery, you may pay the mana cost of a locked door to unlock it.) // Other permanents you control have hexproof.
+(You may cast either half. That door unlocks on the battlefield. As a sorcery, you may pay the mana cost of a locked door to unlock it.)</t>
         </is>
       </c>
     </row>
@@ -2440,13 +2935,24 @@
           <t>VOC</t>
         </is>
       </c>
-      <c r="I46">
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J46">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Reconnaissance%20Mission&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>1.50$</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Whenever a creature you control deals combat damage to a player, you may draw a card.
+Cycling {2} ({2}, Discard this card: Draw a card.)</t>
         </is>
       </c>
     </row>
@@ -2483,13 +2989,23 @@
           <t>SOC</t>
         </is>
       </c>
-      <c r="I47">
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J47">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Tocasia%27s%20Welcome&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t>0.58$</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Whenever one or more creatures you control with mana value 3 or less enter, draw a card. This ability triggers only once each turn.</t>
         </is>
       </c>
     </row>
@@ -2526,13 +3042,23 @@
           <t>ZNC</t>
         </is>
       </c>
-      <c r="I48">
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J48">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Military%20Intelligence&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>0.36$</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Whenever you attack with two or more creatures, draw a card.</t>
         </is>
       </c>
     </row>
@@ -2569,13 +3095,23 @@
           <t>SOC</t>
         </is>
       </c>
-      <c r="I49">
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J49">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Path%20to%20Exile&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>0.99$</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Exile target creature. Its controller may search their library for a basic land card, put that card onto the battlefield tapped, then shuffle.</t>
         </is>
       </c>
     </row>
@@ -2612,13 +3148,25 @@
           <t>TLA</t>
         </is>
       </c>
-      <c r="I50">
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J50">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Airbender%27s%20Reversal&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>0.26$</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Choose one -
+- Destroy target attacking creature.
+- Airbend target creature you control. (Exile it. While it's exiled, its owner may cast it for {2} rather than its mana cost.)</t>
         </is>
       </c>
     </row>
@@ -2655,13 +3203,23 @@
           <t>SOS</t>
         </is>
       </c>
-      <c r="I51">
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J51">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Essence%20Scatter&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t>0.20$</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Counter target creature spell.</t>
         </is>
       </c>
     </row>
@@ -2698,13 +3256,23 @@
           <t>TMT</t>
         </is>
       </c>
-      <c r="I52">
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J52">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Negate&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t>0.27$</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Counter target noncreature spell.</t>
         </is>
       </c>
     </row>
@@ -2741,13 +3309,23 @@
           <t>TDC</t>
         </is>
       </c>
-      <c r="I53">
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J53">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Stroke%20of%20Midnight&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="K53" t="inlineStr">
         <is>
           <t>0.34$</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Destroy target nonland permanent. Its controller creates a 1/1 white Human creature token.</t>
         </is>
       </c>
     </row>
@@ -2784,13 +3362,23 @@
           <t>CMR</t>
         </is>
       </c>
-      <c r="I54">
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J54">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=White%20Sun%27s%20Zenith&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t>0.32$</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Create X 2/2 white Cat creature tokens. Shuffle White Sun's Zenith into its owner's library.</t>
         </is>
       </c>
     </row>
@@ -2827,13 +3415,24 @@
           <t>TMT</t>
         </is>
       </c>
-      <c r="I55">
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J55">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=The%20Last%20Ronin%27s%20Technique&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J55" t="inlineStr">
+      <c r="K55" t="inlineStr">
         <is>
           <t>0.25$</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Sneak {1}{W} (You may cast this spell for {1}{W} if you also return an unblocked attacker you control to hand during the declare blockers step.)
+Create three 1/1 white Ninja Turtle Spirit creature tokens. If this spell's sneak cost was paid, they enter tapped and attacking.</t>
         </is>
       </c>
     </row>
@@ -2870,13 +3469,23 @@
           <t>LCC</t>
         </is>
       </c>
-      <c r="I56">
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J56">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Generous%20Gift&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t>1.62$</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Destroy target permanent. Its controller creates a 3/3 green Elephant creature token.</t>
         </is>
       </c>
     </row>
@@ -2913,13 +3522,23 @@
           <t>SOC</t>
         </is>
       </c>
-      <c r="I57">
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J57">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Swords%20to%20Plowshares&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="K57" t="inlineStr">
         <is>
           <t>1.33$</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Exile target creature. Its controller gains life equal to its power.</t>
         </is>
       </c>
     </row>
@@ -2956,13 +3575,24 @@
           <t>MOC</t>
         </is>
       </c>
-      <c r="I58">
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J58">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Path%20of%20the%20Ghosthunter&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J58" t="inlineStr">
+      <c r="K58" t="inlineStr">
         <is>
           <t>0.30$</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Create X 1/1 white Spirit creature tokens with flying.
+Will of the Planeswalkers - Starting with you, each player votes for planeswalk or chaos. If planeswalk gets more votes, planeswalk. If chaos gets more votes or the vote is tied, chaos ensues.</t>
         </is>
       </c>
     </row>
@@ -2999,13 +3629,23 @@
           <t>LTR</t>
         </is>
       </c>
-      <c r="I59">
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J59">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=The%20Battle%20of%20Bywater&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J59" t="inlineStr">
+      <c r="K59" t="inlineStr">
         <is>
           <t>3.08$</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Destroy all creatures with power 3 or greater. Then create a Food token for each creature you control. (It's an artifact with "{2}, {T}, Sacrifice this token: You gain 3 life.")</t>
         </is>
       </c>
     </row>
@@ -3042,13 +3682,25 @@
           <t>MH3</t>
         </is>
       </c>
-      <c r="I60">
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J60">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Decree%20of%20Justice&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J60" t="inlineStr">
+      <c r="K60" t="inlineStr">
         <is>
           <t>0.27$</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Create X 4/4 white Angel creature tokens with flying.
+Cycling {2}{W} ({2}{W}, Discard this card: Draw a card.)
+When you cycle this card, you may pay {X}. If you do, create X 1/1 white Soldier creature tokens.</t>
         </is>
       </c>
     </row>
@@ -3085,13 +3737,23 @@
           <t>TDC</t>
         </is>
       </c>
-      <c r="I61">
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J61">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Expel%20the%20Interlopers&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="K61" t="inlineStr">
         <is>
           <t>0.28$</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Choose a number between 0 and 10. Destroy all creatures with power greater than or equal to the chosen number.</t>
         </is>
       </c>
     </row>
@@ -3128,13 +3790,23 @@
           <t>MKC</t>
         </is>
       </c>
-      <c r="I62">
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J62">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Fell%20the%20Mighty&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="K62" t="inlineStr">
         <is>
           <t>0.22$</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Destroy all creatures with power greater than target creature's power.</t>
         </is>
       </c>
     </row>
@@ -3171,13 +3843,24 @@
           <t>MKC</t>
         </is>
       </c>
-      <c r="I63">
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J63">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Dusk%20%2F%2F%20Dawn&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J63" t="inlineStr">
+      <c r="K63" t="inlineStr">
         <is>
           <t>0.32$</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Destroy all creatures with power 3 or greater. // Aftermath (Cast this spell only from your graveyard. Then exile it.)
+Return all creature cards with power 2 or less from your graveyard to your hand.</t>
         </is>
       </c>
     </row>
@@ -3214,13 +3897,24 @@
           <t>EOC</t>
         </is>
       </c>
-      <c r="I64">
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J64">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Glacial%20Fortress&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J64" t="inlineStr">
+      <c r="K64" t="inlineStr">
         <is>
           <t>0.33$</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>This land enters tapped unless you control a Plains or an Island.
+{T}: Add {W} or {U}.</t>
         </is>
       </c>
     </row>
@@ -3257,13 +3951,24 @@
           <t>DMU</t>
         </is>
       </c>
-      <c r="I65">
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J65">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Idyllic%20Beachfront&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J65" t="inlineStr">
+      <c r="K65" t="inlineStr">
         <is>
           <t>0.26$</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>({T}: Add {W} or {U}.)
+This land enters tapped.</t>
         </is>
       </c>
     </row>
@@ -3300,13 +4005,25 @@
           <t>EOC</t>
         </is>
       </c>
-      <c r="I66">
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J66">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Irrigated%20Farmland&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J66" t="inlineStr">
+      <c r="K66" t="inlineStr">
         <is>
           <t>0.17$</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>({T}: Add {W} or {U}.)
+This land enters tapped.
+Cycling {2} ({2}, Discard this card: Draw a card.)</t>
         </is>
       </c>
     </row>
@@ -3343,11 +4060,21 @@
           <t>HOB</t>
         </is>
       </c>
-      <c r="I67">
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J67">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Island&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>({T}: Add {U}.)</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="270" customHeight="1">
       <c r="A68" t="inlineStr">
@@ -3382,13 +4109,25 @@
           <t>TLA</t>
         </is>
       </c>
-      <c r="I68">
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J68">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=North%20Pole%20Gates&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J68" t="inlineStr">
+      <c r="K68" t="inlineStr">
         <is>
           <t>0.24$</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>This land enters tapped.
+{T}: Add {W} or {U}.
+{4}, {T}, Sacrifice this land: Draw a card.</t>
         </is>
       </c>
     </row>
@@ -3425,11 +4164,21 @@
           <t>HOB</t>
         </is>
       </c>
-      <c r="I69">
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J69">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Plains&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>({T}: Add {W}.)</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="270" customHeight="1">
       <c r="A70" t="inlineStr">
@@ -3464,13 +4213,24 @@
           <t>CMM</t>
         </is>
       </c>
-      <c r="I70">
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J70">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Port%20Town&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J70" t="inlineStr">
+      <c r="K70" t="inlineStr">
         <is>
           <t>0.22$</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>As this land enters, you may reveal a Plains or Island card from your hand. If you don't, this land enters tapped.
+{T}: Add {W} or {U}.</t>
         </is>
       </c>
     </row>
@@ -3507,13 +4267,24 @@
           <t>TDC</t>
         </is>
       </c>
-      <c r="I71">
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J71">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Prairie%20Stream&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J71" t="inlineStr">
+      <c r="K71" t="inlineStr">
         <is>
           <t>0.26$</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>({T}: Add {W} or {U}.)
+This land enters tapped unless you control two or more basic lands.</t>
         </is>
       </c>
     </row>
@@ -3550,13 +4321,23 @@
           <t>EOC</t>
         </is>
       </c>
-      <c r="I72">
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J72">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Skycloud%20Expanse&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J72" t="inlineStr">
+      <c r="K72" t="inlineStr">
         <is>
           <t>0.27$</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>{1}, {T}: Add {W}{U}.</t>
         </is>
       </c>
     </row>
@@ -3593,13 +4374,25 @@
           <t>EOC</t>
         </is>
       </c>
-      <c r="I73">
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J73">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Temple%20of%20Enlightenment&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J73" t="inlineStr">
+      <c r="K73" t="inlineStr">
         <is>
           <t>0.26$</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>This land enters tapped.
+When this land enters, scry 1. (Look at the top card of your library. You may put that card on the bottom.)
+{T}: Add {W} or {U}.</t>
         </is>
       </c>
     </row>
@@ -3636,13 +4429,24 @@
           <t>ECC</t>
         </is>
       </c>
-      <c r="I74">
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J74">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Thriving%20Heath&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J74" t="inlineStr">
+      <c r="K74" t="inlineStr">
         <is>
           <t>0.23$</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>This land enters tapped. As it enters, choose a color other than white.
+{T}: Add {W} or one mana of the chosen color.</t>
         </is>
       </c>
     </row>
@@ -3679,13 +4483,24 @@
           <t>TMC</t>
         </is>
       </c>
-      <c r="I75">
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J75">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Thriving%20Isle&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J75" t="inlineStr">
+      <c r="K75" t="inlineStr">
         <is>
           <t>0.29$</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>This land enters tapped. As it enters, choose a color other than blue.
+{T}: Add {U} or one mana of the chosen color.</t>
         </is>
       </c>
     </row>
@@ -3722,13 +4537,23 @@
           <t>SOC</t>
         </is>
       </c>
-      <c r="I76">
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J76">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Command%20Tower&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J76" t="inlineStr">
+      <c r="K76" t="inlineStr">
         <is>
           <t>0.34$</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>{T}: Add one mana of any color in your commander's color identity.</t>
         </is>
       </c>
     </row>
@@ -3767,13 +4592,25 @@
           <t>ECL</t>
         </is>
       </c>
-      <c r="I77">
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J77">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Stalactite%20Dagger&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J77" t="inlineStr">
+      <c r="K77" t="inlineStr">
         <is>
           <t>0.23$</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>When this Equipment enters, create a 1/1 colorless Shapeshifter creature token with changeling. (It's every creature type.)
+Equipped creature gets +1/+1 and is all creature types.
+Equip {2} ({2}: Attach to target creature you control. Equip only as a sorcery.)</t>
         </is>
       </c>
     </row>
@@ -3812,13 +4649,24 @@
           <t>FIN</t>
         </is>
       </c>
-      <c r="I78">
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J78">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Magitek%20Armor&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J78" t="inlineStr">
+      <c r="K78" t="inlineStr">
         <is>
           <t>0.06$</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>When this Vehicle enters, create a 1/1 colorless Hero creature token.
+Crew 1 (Tap any number of creatures you control with total power 1 or more: This Vehicle becomes an artifact creature until end of turn.)</t>
         </is>
       </c>
     </row>
@@ -3857,13 +4705,25 @@
           <t>TDM</t>
         </is>
       </c>
-      <c r="I79">
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J79">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Stormbeacon%20Blade&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J79" t="inlineStr">
+      <c r="K79" t="inlineStr">
         <is>
           <t>0.25$</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Equipped creature gets +3/+0.
+Whenever equipped creature attacks, draw a card if you control three or more attacking creatures.
+Equip {2} ({2}: Attach to target creature you control. Equip only as a sorcery.)</t>
         </is>
       </c>
     </row>
@@ -3902,13 +4762,24 @@
           <t>FDN</t>
         </is>
       </c>
-      <c r="I80">
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="J80">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Guarded%20Heir&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J80" t="inlineStr">
+      <c r="K80" t="inlineStr">
         <is>
           <t>0.11$</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Lifelink (Damage dealt by this creature also causes you to gain that much life.)
+When this creature enters, create two 3/3 white Knight creature tokens.</t>
         </is>
       </c>
     </row>
@@ -3947,13 +4818,23 @@
           <t>TLA</t>
         </is>
       </c>
-      <c r="I81">
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J81">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Kyoshi%20Warriors&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J81" t="inlineStr">
+      <c r="K81" t="inlineStr">
         <is>
           <t>0.12$</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>When this creature enters, create a 1/1 white Ally creature token.</t>
         </is>
       </c>
     </row>
@@ -3992,13 +4873,23 @@
           <t>TLA</t>
         </is>
       </c>
-      <c r="I82">
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J82">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Gather%20the%20White%20Lotus&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J82" t="inlineStr">
+      <c r="K82" t="inlineStr">
         <is>
           <t>0.15$</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Create a 1/1 white Ally creature token for each Plains you control. Scry 2. (Look at the top two cards of your library, then put any number of them on the bottom and the rest on top in any order.)</t>
         </is>
       </c>
     </row>
@@ -4037,13 +4928,24 @@
           <t>LCC</t>
         </is>
       </c>
-      <c r="I83">
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J83">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=March%20of%20the%20Canonized&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J83" t="inlineStr">
+      <c r="K83" t="inlineStr">
         <is>
           <t>0.31$</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>When this enchantment enters, create X 1/1 white Vampire creature tokens with lifelink.
+At the beginning of your upkeep, if your devotion to white and black is seven or greater, create a 4/3 white and black Vampire Demon creature token with flying.</t>
         </is>
       </c>
     </row>
@@ -4082,13 +4984,23 @@
           <t>TDC</t>
         </is>
       </c>
-      <c r="I84">
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J84">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Release%20the%20Dogs&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J84" t="inlineStr">
+      <c r="K84" t="inlineStr">
         <is>
           <t>0.34$</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Create four 1/1 white Dog creature tokens.</t>
         </is>
       </c>
     </row>
@@ -4127,13 +5039,24 @@
           <t>OTC</t>
         </is>
       </c>
-      <c r="I85">
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J85">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Prismatic%20Lens&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J85" t="inlineStr">
+      <c r="K85" t="inlineStr">
         <is>
           <t>0.41$</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>{T}: Add {C}.
+{1}, {T}: Add one mana of any color.</t>
         </is>
       </c>
     </row>
@@ -4172,13 +5095,25 @@
           <t>DSK</t>
         </is>
       </c>
-      <c r="I86">
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J86">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Cursed%20Windbreaker&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J86" t="inlineStr">
+      <c r="K86" t="inlineStr">
         <is>
           <t>0.16$</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>When this Equipment enters, manifest dread, then attach this Equipment to that creature. (Look at the top two cards of your library. Put one onto the battlefield face down as a 2/2 creature and the other into your graveyard. Turn it face up any time for its mana cost if it's a creature card.)
+Equipped creature has flying.
+Equip {3}</t>
         </is>
       </c>
     </row>
@@ -4217,13 +5152,25 @@
           <t>TLA</t>
         </is>
       </c>
-      <c r="I87">
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J87">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Fire%20Nation%20Warship&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J87" t="inlineStr">
+      <c r="K87" t="inlineStr">
         <is>
           <t>0.13$</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Reach
+When this Vehicle dies, create a Clue token. (It's an artifact with "{2}, Sacrifice this token: Draw a card.")
+Crew 2 (Tap any number of creatures you control with total power 2 or more: This Vehicle becomes an artifact creature until end of turn.)</t>
         </is>
       </c>
     </row>
@@ -4262,13 +5209,23 @@
           <t>SOS</t>
         </is>
       </c>
-      <c r="I88">
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J88">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Quick%20Study&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J88" t="inlineStr">
+      <c r="K88" t="inlineStr">
         <is>
           <t>0.18$</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Draw two cards.</t>
         </is>
       </c>
     </row>
@@ -4307,13 +5264,23 @@
           <t>FDN</t>
         </is>
       </c>
-      <c r="I89">
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J89">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Refute&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J89" t="inlineStr">
+      <c r="K89" t="inlineStr">
         <is>
           <t>0.29$</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Counter target spell. Draw a card, then discard a card.</t>
         </is>
       </c>
     </row>
@@ -4352,13 +5319,23 @@
           <t>FIN</t>
         </is>
       </c>
-      <c r="I90">
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="J90">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=The%20Crystal%27s%20Chosen&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J90" t="inlineStr">
+      <c r="K90" t="inlineStr">
         <is>
           <t>0.15$</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Create four 1/1 colorless Hero creature tokens. Then put a +1/+1 counter on each creature you control.</t>
         </is>
       </c>
     </row>
@@ -4397,13 +5374,24 @@
           <t>TLA</t>
         </is>
       </c>
-      <c r="I91">
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J91">
         <f>IMAGE("https://api.scryfall.com/cards/named?exact=Team%20Avatar&amp;format=image&amp;version=normal")</f>
         <v/>
       </c>
-      <c r="J91" t="inlineStr">
+      <c r="K91" t="inlineStr">
         <is>
           <t>0.18$</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Whenever a creature you control attacks alone, it gets +X/+X until end of turn, where X is the number of creatures you control.
+{2}{W}, Discard this card: It deals damage equal to the number of creatures you control to target creature.</t>
         </is>
       </c>
     </row>
@@ -4413,8 +5401,8 @@
           <t>Total Cost (Have Physical Copy = false)</t>
         </is>
       </c>
-      <c r="J93" s="2">
-        <f>SUMPRODUCT(--(LOWER(TEXT($C$2:$C$91,"@"))="false"),IFERROR(VALUE(SUBSTITUTE($J$2:$J$91,"$","")),0))</f>
+      <c r="K93" s="2">
+        <f>SUMPRODUCT(--(LOWER(TEXT($C$2:$C$91,"@"))="false"),IFERROR(VALUE(SUBSTITUTE($K$2:$K$91,"$","")),0))</f>
         <v/>
       </c>
     </row>

</xml_diff>